<commit_message>
ultimos cambios en estrategia
</commit_message>
<xml_diff>
--- a/salidas/estrategia/estrategia.xlsx
+++ b/salidas/estrategia/estrategia.xlsx
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:S7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -581,6 +581,11 @@
           <t>r2_mercado</t>
         </is>
       </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>treynor</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -639,6 +644,9 @@
       <c r="R2" t="n">
         <v>0.06796554051072923</v>
       </c>
+      <c r="S2" t="n">
+        <v>0.3711162596165761</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -697,6 +705,9 @@
       <c r="R3" t="n">
         <v>0.0683258700673357</v>
       </c>
+      <c r="S3" t="n">
+        <v>0.3433173475405074</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -755,6 +766,9 @@
       <c r="R4" t="n">
         <v>0.7132663660388847</v>
       </c>
+      <c r="S4" t="n">
+        <v>0.2112164926203405</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -813,6 +827,9 @@
       <c r="R5" t="n">
         <v>0.7317293636814536</v>
       </c>
+      <c r="S5" t="n">
+        <v>0.1922454266203953</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -871,6 +888,9 @@
       <c r="R6" t="n">
         <v>0.9488524918702514</v>
       </c>
+      <c r="S6" t="n">
+        <v>0.178760485889209</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -928,6 +948,9 @@
       </c>
       <c r="R7" t="n">
         <v>1</v>
+      </c>
+      <c r="S7" t="n">
+        <v>0.1127582869179651</v>
       </c>
     </row>
   </sheetData>
@@ -1742,7 +1765,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S13"/>
+  <dimension ref="A1:T13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1841,6 +1864,11 @@
           <t>r2_mercado</t>
         </is>
       </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>treynor</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1904,6 +1932,9 @@
       <c r="S2" t="n">
         <v>0.1246198581738734</v>
       </c>
+      <c r="T2" t="n">
+        <v>0.1686453315229118</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1967,6 +1998,9 @@
       <c r="S3" t="n">
         <v>0.125152210589681</v>
       </c>
+      <c r="T3" t="n">
+        <v>0.1498087784662686</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2030,6 +2064,9 @@
       <c r="S4" t="n">
         <v>0.8203840000664738</v>
       </c>
+      <c r="T4" t="n">
+        <v>0.1560982473883528</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2093,6 +2130,9 @@
       <c r="S5" t="n">
         <v>0.7462453084422909</v>
       </c>
+      <c r="T5" t="n">
+        <v>0.1676979095438464</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2156,6 +2196,9 @@
       <c r="S6" t="n">
         <v>0.9805578583026384</v>
       </c>
+      <c r="T6" t="n">
+        <v>0.1588831049385718</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2219,6 +2262,9 @@
       <c r="S7" t="n">
         <v>1</v>
       </c>
+      <c r="T7" t="n">
+        <v>0.1075724093418538</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2282,6 +2328,9 @@
       <c r="S8" t="n">
         <v>0.05165626375570742</v>
       </c>
+      <c r="T8" t="n">
+        <v>0.5951118651348509</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2345,6 +2394,9 @@
       <c r="S9" t="n">
         <v>0.05207195295118094</v>
       </c>
+      <c r="T9" t="n">
+        <v>0.5580194457492761</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2408,6 +2460,9 @@
       <c r="S10" t="n">
         <v>0.678057867661352</v>
       </c>
+      <c r="T10" t="n">
+        <v>0.2659612890186061</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2471,6 +2526,9 @@
       <c r="S11" t="n">
         <v>0.7281886966845814</v>
       </c>
+      <c r="T11" t="n">
+        <v>0.2193644630493391</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2534,6 +2592,9 @@
       <c r="S12" t="n">
         <v>0.9353793440588587</v>
       </c>
+      <c r="T12" t="n">
+        <v>0.196424861029765</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2596,6 +2657,9 @@
       </c>
       <c r="S13" t="n">
         <v>1</v>
+      </c>
+      <c r="T13" t="n">
+        <v>0.1179441644940764</v>
       </c>
     </row>
   </sheetData>
@@ -11899,7 +11963,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12001,34 +12065,46 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>dif_media_anualizada / t_stat_dif</t>
+          <t>treynor</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Diferencia mensual contra la pasiva (x12) y su t pareada</t>
+          <t>Rendimiento en exceso medio anualizado / beta_mercado</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Cuantiles</t>
+          <t>dif_media_anualizada / t_stat_dif</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Rendimiento real promedio por quintil del rendimiento esperado; Q1 = menor E[R]</t>
+          <t>Diferencia mensual contra la pasiva (x12) y su t pareada</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>Cuantiles</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Rendimiento real promedio por quintil del rendimiento esperado; Q1 = menor E[R]</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>Sesgo</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>El modelo se eligió con el mismo periodo que se usa aquí; el desempeño es en-muestra respecto a esa elección</t>
         </is>

</xml_diff>